<commit_message>
:feet Tool Selector 및 공정능력,Uutlier,동등성 검정 Update
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\open_minitab\multi_page\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\open_minitab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27DECB79-6F4E-47AF-A3DF-DE31C77753E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5822BF80-3212-457B-8A5C-4C7819FEEEDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{CF082BDA-F820-4619-809B-E96ADB11BB0D}"/>
+    <workbookView xWindow="885" yWindow="3382" windowWidth="16200" windowHeight="9308" xr2:uid="{CF082BDA-F820-4619-809B-E96ADB11BB0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -491,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB4B5083-3734-4CE3-AAE9-E47C2579A957}">
-  <dimension ref="B1:Q27"/>
+  <dimension ref="B1:Q38"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.6">
@@ -524,11 +524,11 @@
       </c>
       <c r="H2">
         <f ca="1">RAND()</f>
-        <v>0.18877362557319788</v>
+        <v>0.21479012108842876</v>
       </c>
       <c r="I2">
         <f ca="1">F2+(H2+10)^3</f>
-        <v>1072.7078791624026</v>
+        <v>1080.8309895084885</v>
       </c>
       <c r="K2" t="s">
         <v>7</v>
@@ -553,11 +553,11 @@
       </c>
       <c r="H3">
         <f ca="1">RAND()</f>
-        <v>0.37041021812046637</v>
+        <v>0.49742323583185621</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I41" ca="1" si="1">F3+(H3+10)^3</f>
-        <v>1132.2899989902223</v>
+        <f t="shared" ref="I3:I21" ca="1" si="1">F3+(H3+10)^3</f>
+        <v>1173.7729443852554</v>
       </c>
       <c r="K3">
         <v>25.8</v>
@@ -600,7 +600,7 @@
       </c>
       <c r="H4">
         <f t="shared" ref="H4:H21" ca="1" si="2">RAND()</f>
-        <v>0.47640065527988207</v>
+        <v>0.55176946729643495</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -646,11 +646,11 @@
       </c>
       <c r="H5">
         <f t="shared" ca="1" si="2"/>
-        <v>0.30278008458202399</v>
+        <v>0.76718760066112002</v>
       </c>
       <c r="I5">
         <f t="shared" ca="1" si="1"/>
-        <v>1110.6120563634993</v>
+        <v>1265.2651334707853</v>
       </c>
       <c r="K5">
         <v>26.1</v>
@@ -693,11 +693,11 @@
       </c>
       <c r="H6">
         <f t="shared" ca="1" si="2"/>
-        <v>0.63880313699693458</v>
+        <v>6.4894968820847332E-2</v>
       </c>
       <c r="I6">
         <f t="shared" ca="1" si="1"/>
-        <v>1218.1437005775849</v>
+        <v>1033.595104651482</v>
       </c>
       <c r="K6">
         <v>22.9</v>
@@ -734,7 +734,7 @@
       </c>
       <c r="H7">
         <f t="shared" ca="1" si="2"/>
-        <v>0.61411163074765729</v>
+        <v>0.38652757025786488</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -774,11 +774,11 @@
       </c>
       <c r="H8">
         <f t="shared" ca="1" si="2"/>
-        <v>0.48964511284642265</v>
+        <v>0.80563145171893114</v>
       </c>
       <c r="I8">
         <f t="shared" ca="1" si="1"/>
-        <v>1166.2034975098361</v>
+        <v>1273.68358527333</v>
       </c>
       <c r="K8">
         <v>27.3</v>
@@ -815,11 +815,11 @@
       </c>
       <c r="H9">
         <f t="shared" ca="1" si="2"/>
-        <v>0.81078698850510256</v>
+        <v>0.18043232939052323</v>
       </c>
       <c r="I9">
         <f t="shared" ca="1" si="1"/>
-        <v>1282.4903543083904</v>
+        <v>1074.1122477052641</v>
       </c>
       <c r="K9">
         <v>24</v>
@@ -856,11 +856,11 @@
       </c>
       <c r="H10">
         <f t="shared" ca="1" si="2"/>
-        <v>0.23718806831417538</v>
+        <v>0.36726223748647668</v>
       </c>
       <c r="I10">
         <f t="shared" ca="1" si="1"/>
-        <v>1091.8575096557529</v>
+        <v>1133.2746546786968</v>
       </c>
       <c r="K10">
         <v>24.5</v>
@@ -894,11 +894,11 @@
       </c>
       <c r="H11">
         <f t="shared" ca="1" si="2"/>
-        <v>1.3663020837441753E-2</v>
+        <v>0.32725050837615277</v>
       </c>
       <c r="I11">
         <f t="shared" ca="1" si="1"/>
-        <v>1018.1045091459719</v>
+        <v>1115.4229855742278</v>
       </c>
       <c r="K11">
         <v>23.9</v>
@@ -929,7 +929,7 @@
       </c>
       <c r="H12">
         <f t="shared" ca="1" si="2"/>
-        <v>0.58382575591158614</v>
+        <v>0.97100913190257598</v>
       </c>
       <c r="I12">
         <v>10</v>
@@ -963,11 +963,11 @@
       </c>
       <c r="H13">
         <f t="shared" ca="1" si="2"/>
-        <v>0.71302558479290279</v>
+        <v>0.9514711226819681</v>
       </c>
       <c r="I13">
         <f t="shared" ca="1" si="1"/>
-        <v>1251.5223460928955</v>
+        <v>1335.4616199593415</v>
       </c>
       <c r="K13">
         <v>24.3</v>
@@ -998,11 +998,11 @@
       </c>
       <c r="H14">
         <f t="shared" ca="1" si="2"/>
-        <v>0.29763014092284268</v>
+        <v>0.49516099187242579</v>
       </c>
       <c r="I14">
         <f t="shared" ca="1" si="1"/>
-        <v>1115.9729184797739</v>
+        <v>1180.025235552484</v>
       </c>
       <c r="K14">
         <v>24.6</v>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="H15">
         <f t="shared" ca="1" si="2"/>
-        <v>0.48967383077223448</v>
+        <v>0.3067052507846546</v>
       </c>
       <c r="I15">
         <v>20</v>
@@ -1055,17 +1055,17 @@
       </c>
       <c r="H16">
         <f t="shared" ca="1" si="2"/>
-        <v>0.79525908593887462</v>
+        <v>0.28568206964421783</v>
       </c>
       <c r="I16">
         <f t="shared" ca="1" si="1"/>
-        <v>1271.053787476196</v>
+        <v>1101.1763639671515</v>
       </c>
       <c r="K16">
         <v>25.5</v>
       </c>
     </row>
-    <row r="17" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.6">
       <c r="E17">
         <v>16</v>
       </c>
@@ -1078,17 +1078,17 @@
       </c>
       <c r="H17">
         <f t="shared" ca="1" si="2"/>
-        <v>0.39722184187805332</v>
+        <v>0.3329717822406395</v>
       </c>
       <c r="I17">
         <f t="shared" ca="1" si="1"/>
-        <v>1139.9627840378203</v>
+        <v>1119.254557555925</v>
       </c>
       <c r="K17">
         <v>28.1</v>
       </c>
     </row>
-    <row r="18" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.6">
       <c r="E18">
         <v>16</v>
       </c>
@@ -1101,17 +1101,17 @@
       </c>
       <c r="H18">
         <f t="shared" ca="1" si="2"/>
-        <v>5.1664670909286614E-2</v>
+        <v>0.67772946552946201</v>
       </c>
       <c r="I18">
         <f t="shared" ca="1" si="1"/>
-        <v>1028.5796163247051</v>
+        <v>1230.4096493319878</v>
       </c>
       <c r="K18">
         <v>24.8</v>
       </c>
     </row>
-    <row r="19" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.6">
       <c r="E19">
         <v>13</v>
       </c>
@@ -1124,17 +1124,17 @@
       </c>
       <c r="H19">
         <f t="shared" ca="1" si="2"/>
-        <v>0.34561031205019577</v>
+        <v>0.33656422114564</v>
       </c>
       <c r="I19">
         <f t="shared" ca="1" si="1"/>
-        <v>1125.3077701868422</v>
+        <v>1122.4056550643563</v>
       </c>
       <c r="K19">
         <v>23.5</v>
       </c>
     </row>
-    <row r="20" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.6">
       <c r="E20">
         <v>14</v>
       </c>
@@ -1147,17 +1147,17 @@
       </c>
       <c r="H20">
         <f t="shared" ca="1" si="2"/>
-        <v>5.2691712520011258E-2</v>
+        <v>0.42541842211586778</v>
       </c>
       <c r="I20">
         <f t="shared" ca="1" si="1"/>
-        <v>1030.8909525471961</v>
+        <v>1148.1319442318077</v>
       </c>
       <c r="K20">
         <v>26.3</v>
       </c>
     </row>
-    <row r="21" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.6">
       <c r="E21">
         <v>12</v>
       </c>
@@ -1170,22 +1170,22 @@
       </c>
       <c r="H21">
         <f t="shared" ca="1" si="2"/>
-        <v>0.43046566252665941</v>
+        <v>0.649271760194989</v>
       </c>
       <c r="I21">
         <f t="shared" ca="1" si="1"/>
-        <v>1147.7784849392633</v>
+        <v>1220.7018456059081</v>
       </c>
       <c r="K21">
         <v>25.4</v>
       </c>
     </row>
-    <row r="22" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.6">
       <c r="K22">
         <v>25.5</v>
       </c>
     </row>
-    <row r="23" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.6">
       <c r="E23">
         <f>AVERAGE(E2:E21)</f>
         <v>15.15</v>
@@ -1202,24 +1202,123 @@
         <v>23.9</v>
       </c>
     </row>
-    <row r="24" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.6">
       <c r="K24">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.6">
       <c r="K25">
         <v>24.8</v>
       </c>
     </row>
-    <row r="26" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.6">
       <c r="K26">
         <v>22.9</v>
       </c>
     </row>
-    <row r="27" spans="5:11" x14ac:dyDescent="0.6">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.6">
       <c r="K27">
         <v>25.4</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.6">
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.6">
+      <c r="B29">
+        <f t="shared" ref="B29:B37" si="3">B28*2</f>
+        <v>2</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.6">
+      <c r="B30">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="C30">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.6">
+      <c r="B31">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.6">
+      <c r="B32">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="C32">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.6">
+      <c r="B33">
+        <f t="shared" si="3"/>
+        <v>32</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.6">
+      <c r="B34">
+        <f t="shared" si="3"/>
+        <v>64</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.6">
+      <c r="B35">
+        <f t="shared" si="3"/>
+        <v>128</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.6">
+      <c r="B36">
+        <f t="shared" si="3"/>
+        <v>256</v>
+      </c>
+      <c r="C36">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.6">
+      <c r="B37">
+        <f t="shared" si="3"/>
+        <v>512</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.6">
+      <c r="B38">
+        <f>_xlfn.STDEV.S(B28:B37)</f>
+        <v>164.94851048466947</v>
+      </c>
+      <c r="C38">
+        <f>_xlfn.STDEV.S(C28:C37)</f>
+        <v>0.81649658092772603</v>
       </c>
     </row>
   </sheetData>

</xml_diff>